<commit_message>
organize damper series and functions
</commit_message>
<xml_diff>
--- a/docs/damping_curve_MRAx0.xlsx
+++ b/docs/damping_curve_MRAx0.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="115">
   <si>
     <t>Astral · LSC Sweep</t>
   </si>
@@ -299,6 +299,93 @@
     <t>Astral · HSC Sweep</t>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
+  <si>
+    <t>CTM Racing · MRAx0 · Damping Calculator</t>
+  </si>
+  <si>
+    <t>MRA60 / MRA80 · 柏油拉力 · c / C / R 调节与阻尼力计算</t>
+  </si>
+  <si>
+    <t>适用车型</t>
+  </si>
+  <si>
+    <t>当前曲线参数</t>
+  </si>
+  <si>
+    <t>HSbump · 高速增量</t>
+  </si>
+  <si>
+    <t>CTM Racing · MRAx0 · Valving Parameters</t>
+  </si>
+  <si>
+    <t>MRA60 / MRA60 (Mod) / MRA80 · 柏油拉力系列；黄色单元格为可编辑标定。</t>
+  </si>
+  <si>
+    <t>HSbump · 高速增量</t>
+  </si>
+  <si>
+    <t>LSR · R（MRA60）</t>
+  </si>
+  <si>
+    <t>Adjusters · 调节格数</t>
+  </si>
+  <si>
+    <t>LSC · 全系列</t>
+  </si>
+  <si>
+    <t>HSC · 全系列</t>
+  </si>
+  <si>
+    <t>LSR · MRA60</t>
+  </si>
+  <si>
+    <t>LSR · MRA80</t>
+  </si>
+  <si>
+    <t>Sweep 使用 MRA60 的格数；MRA60 (Mod) 同为 40 格回弹，MRA80 为 60 格，适用车型在计算器选择。</t>
+  </si>
+  <si>
+    <t>Model · 基础阻尼模型</t>
+  </si>
+  <si>
+    <t>理论曲线采用连续分段接续假设；仅计算基础阻尼，不包含气体支撑、弹簧、HBS/HRS 或 LRS/DSV。</t>
+  </si>
+  <si>
+    <t>CTM Racing · MRAx0 · LSC Sweep · 读取对应 Sweep 页的阀系选择</t>
+  </si>
+  <si>
+    <t>CTM Racing · MRAx0 · HSC Sweep · 读取对应 Sweep 页的阀系选择</t>
+  </si>
+  <si>
+    <t>CTM Racing · MRAx0 · LSR Sweep · 读取对应 Sweep 页的阀系选择</t>
+  </si>
+  <si>
+    <t>CTM Racing · MRAx0 · Full Sweep · 读取对应 Sweep 页的阀系选择</t>
+  </si>
+  <si>
+    <t>CTM Racing · MRAx0 · LSC Sweep</t>
+  </si>
+  <si>
+    <t>柏油拉力 · Type-A / Type-B 阀系；各页独立选择。</t>
+  </si>
+  <si>
+    <t>CTM Racing · MRAx0 · HSC Sweep</t>
+  </si>
+  <si>
+    <t>柏油拉力 · Type-A / Type-B 阀系；各页独立选择。</t>
+  </si>
+  <si>
+    <t>CTM Racing · MRAx0 · LSR Sweep</t>
+  </si>
+  <si>
+    <t>柏油拉力 · Type-A / Type-B 阀系；各页独立选择。</t>
+  </si>
+  <si>
+    <t>CTM Racing · MRAx0 · Full Sweep</t>
+  </si>
+  <si>
+    <t>柏油拉力 · Type-A / Type-B 阀系；各页独立选择。</t>
+  </si>
 </sst>
 </file>
 
@@ -549,7 +636,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Compression</a:t>
+              <a:t>MRAx0 · LSC Sweep</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1639,7 +1726,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Compression</a:t>
+              <a:t>MRAx0 · HSC Sweep</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2719,7 +2806,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Rebound</a:t>
+              <a:t>MRAx0 · LSR Sweep</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -3792,7 +3879,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Compression (+) / Rebound (−)</a:t>
+              <a:t>MRAx0 · Compression (+) / Rebound (−)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -6124,7 +6211,7 @@
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="24" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
@@ -6167,7 +6254,7 @@
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="25" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
@@ -6200,7 +6287,7 @@
     <row r="6" spans="1:15" ht="23" customHeight="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>47</v>
@@ -6360,7 +6447,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="20" t="s">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="G13" s="20"/>
       <c r="H13" s="20"/>
@@ -6437,7 +6524,7 @@
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="22" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="G16" s="22"/>
       <c r="H16" s="22"/>
@@ -7026,7 +7113,7 @@
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="24" t="s">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
@@ -7069,7 +7156,7 @@
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="25" t="s">
-        <v>3</v>
+        <v>108</v>
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
@@ -7790,7 +7877,7 @@
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="24" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
@@ -7833,7 +7920,7 @@
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="25" t="s">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
@@ -8554,7 +8641,7 @@
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="24" t="s">
-        <v>9</v>
+        <v>111</v>
       </c>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
@@ -8597,7 +8684,7 @@
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="25" t="s">
-        <v>3</v>
+        <v>112</v>
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
@@ -9310,7 +9397,7 @@
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="24" t="s">
-        <v>11</v>
+        <v>113</v>
       </c>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
@@ -9353,7 +9440,7 @@
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="25" t="s">
-        <v>3</v>
+        <v>114</v>
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="25"/>
@@ -10070,7 +10157,7 @@
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="24" t="s">
-        <v>13</v>
+        <v>91</v>
       </c>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
@@ -10089,7 +10176,7 @@
     <row r="3" spans="1:15" ht="23" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="25" t="s">
-        <v>14</v>
+        <v>92</v>
       </c>
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
@@ -10446,7 +10533,7 @@
     <row r="13" spans="1:15" ht="23" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>26</v>
+        <v>93</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>22</v>
@@ -10553,7 +10640,7 @@
     <row r="16" spans="1:15" ht="23" customHeight="1">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>27</v>
+        <v>94</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>19</v>
@@ -10773,7 +10860,7 @@
     <row r="22" spans="1:15" ht="23" customHeight="1">
       <c r="A22" s="1"/>
       <c r="B22" s="20" t="s">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="C22" s="20"/>
       <c r="D22" s="20"/>
@@ -10792,7 +10879,7 @@
     <row r="23" spans="1:15" ht="23" customHeight="1">
       <c r="A23" s="1"/>
       <c r="B23" s="22" t="s">
-        <v>32</v>
+        <v>96</v>
       </c>
       <c r="C23" s="22"/>
       <c r="D23" s="1">
@@ -10800,7 +10887,7 @@
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="23" t="s">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="G23" s="23"/>
       <c r="H23" s="23"/>
@@ -10815,7 +10902,7 @@
     <row r="24" spans="1:15" ht="23" customHeight="1">
       <c r="A24" s="1"/>
       <c r="B24" s="22" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="C24" s="22"/>
       <c r="D24" s="1">
@@ -10836,7 +10923,7 @@
     <row r="25" spans="1:15" ht="23" customHeight="1">
       <c r="A25" s="1"/>
       <c r="B25" s="22" t="s">
-        <v>35</v>
+        <v>98</v>
       </c>
       <c r="C25" s="22"/>
       <c r="D25" s="1">
@@ -10857,7 +10944,7 @@
     <row r="26" spans="1:15" ht="23" customHeight="1">
       <c r="A26" s="1"/>
       <c r="B26" s="22" t="s">
-        <v>36</v>
+        <v>99</v>
       </c>
       <c r="C26" s="22"/>
       <c r="D26" s="1">
@@ -10897,7 +10984,7 @@
     <row r="28" spans="1:15" ht="23" customHeight="1">
       <c r="A28" s="1"/>
       <c r="B28" s="20" t="s">
-        <v>38</v>
+        <v>101</v>
       </c>
       <c r="C28" s="20"/>
       <c r="D28" s="20"/>
@@ -10973,7 +11060,7 @@
     <row r="32" spans="1:15" ht="23" customHeight="1">
       <c r="A32" s="1"/>
       <c r="B32" s="19" t="s">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="C32" s="19"/>
       <c r="D32" s="19"/>
@@ -11191,7 +11278,7 @@
     <row r="1" spans="1:22" ht="22" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="28" t="s">
-        <v>62</v>
+        <v>103</v>
       </c>
       <c r="C1" s="28"/>
       <c r="D1" s="28"/>
@@ -12884,7 +12971,7 @@
     <row r="41" spans="1:22" ht="22" customHeight="1">
       <c r="A41" s="1"/>
       <c r="B41" s="28" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="C41" s="28"/>
       <c r="D41" s="28"/>
@@ -14538,7 +14625,7 @@
     </row>
     <row r="81" spans="2:22" ht="22" customHeight="1">
       <c r="B81" s="29" t="s">
-        <v>78</v>
+        <v>105</v>
       </c>
       <c r="C81" s="29"/>
       <c r="D81" s="29"/>
@@ -16191,7 +16278,7 @@
     </row>
     <row r="121" spans="2:22" ht="22" customHeight="1">
       <c r="B121" s="29" t="s">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="C121" s="29"/>
       <c r="D121" s="29"/>

</xml_diff>

<commit_message>
PREPARE FOR WEIGHT TRANSFER and ARB map
</commit_message>
<xml_diff>
--- a/docs/damping_curve_MRAx0.xlsx
+++ b/docs/damping_curve_MRAx0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B61CA6CC-DDCF-4DFA-8B8D-8D400F134D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C68EC0-C45A-40FC-B563-259B7187135E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculator" sheetId="6" r:id="rId1"/>
@@ -491,20 +491,23 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -512,11 +515,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1506,40 +1506,40 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>182.5</c:v>
+                  <c:v>210</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>360.62</c:v>
+                  <c:v>420</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>532.16999999999996</c:v>
+                  <c:v>630</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>703.72</c:v>
+                  <c:v>840</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>875.27</c:v>
+                  <c:v>984.9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1046.82</c:v>
+                  <c:v>1129.8</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1220.8699999999999</c:v>
+                  <c:v>1274.6999999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1404.92</c:v>
+                  <c:v>1419.6</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1588.97</c:v>
+                  <c:v>1564.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1773.02</c:v>
+                  <c:v>1709.4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1957.0700000000002</c:v>
+                  <c:v>1854.3000000000002</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2141.12</c:v>
+                  <c:v>1999.1999999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1634,40 +1634,40 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>182.5</c:v>
+                  <c:v>210</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>360.62</c:v>
+                  <c:v>420</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>532.16999999999996</c:v>
+                  <c:v>630</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>703.72</c:v>
+                  <c:v>840</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>875.27</c:v>
+                  <c:v>1050</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1046.82</c:v>
+                  <c:v>1194.9000000000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1223.3699999999999</c:v>
+                  <c:v>1339.8</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1444.92</c:v>
+                  <c:v>1484.7</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1666.47</c:v>
+                  <c:v>1629.6</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1888.02</c:v>
+                  <c:v>1774.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2109.5700000000002</c:v>
+                  <c:v>1919.4</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2331.12</c:v>
+                  <c:v>2064.3000000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1762,40 +1762,40 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>182.5</c:v>
+                  <c:v>210</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>360.62</c:v>
+                  <c:v>420</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>532.16999999999996</c:v>
+                  <c:v>630</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>703.72</c:v>
+                  <c:v>840</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>875.27</c:v>
+                  <c:v>1050</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1046.82</c:v>
+                  <c:v>1260</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1218.3699999999999</c:v>
+                  <c:v>1404.9</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1477.42</c:v>
+                  <c:v>1549.8000000000002</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1736.47</c:v>
+                  <c:v>1694.7</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1995.52</c:v>
+                  <c:v>1839.6</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2254.5700000000002</c:v>
+                  <c:v>1984.5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2513.62</c:v>
+                  <c:v>2129.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1890,40 +1890,40 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>182.5</c:v>
+                  <c:v>210</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>360.62</c:v>
+                  <c:v>420</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>532.16999999999996</c:v>
+                  <c:v>630</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>703.72</c:v>
+                  <c:v>840</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>875.27</c:v>
+                  <c:v>1050</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1046.82</c:v>
+                  <c:v>1260</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1218.3699999999999</c:v>
+                  <c:v>1470</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1502.42</c:v>
+                  <c:v>1614.9</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1798.97</c:v>
+                  <c:v>1759.8000000000002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2095.52</c:v>
+                  <c:v>1904.7</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2392.0700000000002</c:v>
+                  <c:v>2049.6000000000004</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2688.62</c:v>
+                  <c:v>2194.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2018,40 +2018,40 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>182.5</c:v>
+                  <c:v>210</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>360.62</c:v>
+                  <c:v>420</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>532.16999999999996</c:v>
+                  <c:v>630</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>703.72</c:v>
+                  <c:v>840</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>875.27</c:v>
+                  <c:v>1050</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1046.82</c:v>
+                  <c:v>1260</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1218.3699999999999</c:v>
+                  <c:v>1470</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1519.92</c:v>
+                  <c:v>1680</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1853.97</c:v>
+                  <c:v>1824.9</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2188.02</c:v>
+                  <c:v>1969.8</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2522.0700000000006</c:v>
+                  <c:v>2114.6999999999998</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2856.12</c:v>
+                  <c:v>2259.6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4934,7 +4934,7 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="22" t="s">
         <v>58</v>
       </c>
       <c r="C2" s="20"/>
@@ -4977,17 +4977,17 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -5018,13 +5018,13 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -5067,11 +5067,11 @@
       </c>
       <c r="G8" s="20"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="26">
+      <c r="I8" s="24">
         <f>IF(C18="OK",Samples!F165*MIN(C10,Samples!G165)+Samples!I165*MAX(0,C10-Samples!G165)+Samples!J165*MAX(0,C10-Samples!K165),"检查输入")</f>
         <v>1736.47</v>
       </c>
-      <c r="J8" s="26"/>
+      <c r="J8" s="24"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -5114,11 +5114,11 @@
       </c>
       <c r="G10" s="20"/>
       <c r="H10" s="20"/>
-      <c r="I10" s="26">
+      <c r="I10" s="24">
         <f>IF(C18="OK",Samples!M165*MIN(C10,Samples!N165)+Samples!P165*MAX(0,C10-Samples!N165),"检查输入")</f>
         <v>1519.2</v>
       </c>
-      <c r="J10" s="26"/>
+      <c r="J10" s="24"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -5170,13 +5170,13 @@
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="22" t="s">
+      <c r="F13" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="21"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
@@ -5484,20 +5484,20 @@
     </row>
     <row r="27" spans="1:15" ht="23" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="27"/>
-      <c r="J27" s="27"/>
-      <c r="K27" s="27"/>
-      <c r="L27" s="27"/>
-      <c r="M27" s="27"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="19"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="19"/>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
     </row>
@@ -5758,17 +5758,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B27:M27"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="F24:H24"/>
-    <mergeCell ref="F13:J13"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F16:H16"/>
-    <mergeCell ref="F17:H17"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="E4:M4"/>
     <mergeCell ref="F6:J6"/>
@@ -5776,6 +5765,17 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="I10:J10"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="B27:M27"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F24:H24"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="6">
@@ -5836,7 +5836,7 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="22" t="s">
         <v>75</v>
       </c>
       <c r="C2" s="20"/>
@@ -5879,17 +5879,17 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -6513,20 +6513,20 @@
     </row>
     <row r="41" spans="1:15" ht="23" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="27" t="s">
+      <c r="B41" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C41" s="27"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="27"/>
-      <c r="J41" s="27"/>
-      <c r="K41" s="27"/>
-      <c r="L41" s="27"/>
-      <c r="M41" s="27"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="19"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="19"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -6600,7 +6600,7 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="22" t="s">
         <v>77</v>
       </c>
       <c r="C2" s="20"/>
@@ -6640,20 +6640,20 @@
         <v>0</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -7277,20 +7277,20 @@
     </row>
     <row r="41" spans="1:15" ht="23" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="27" t="s">
+      <c r="B41" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C41" s="27"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="27"/>
-      <c r="J41" s="27"/>
-      <c r="K41" s="27"/>
-      <c r="L41" s="27"/>
-      <c r="M41" s="27"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="19"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="19"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -7364,7 +7364,7 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="22" t="s">
         <v>79</v>
       </c>
       <c r="C2" s="20"/>
@@ -7407,17 +7407,17 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -8037,20 +8037,20 @@
     </row>
     <row r="41" spans="1:15" ht="23" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="27" t="s">
+      <c r="B41" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C41" s="27"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="27"/>
-      <c r="J41" s="27"/>
-      <c r="K41" s="27"/>
-      <c r="L41" s="27"/>
-      <c r="M41" s="27"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="19"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="19"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -8120,7 +8120,7 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="22" t="s">
         <v>81</v>
       </c>
       <c r="C2" s="20"/>
@@ -8163,17 +8163,17 @@
         <v>1</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
@@ -8793,20 +8793,20 @@
     </row>
     <row r="41" spans="1:15" ht="23" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="27" t="s">
+      <c r="B41" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="C41" s="27"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="27"/>
-      <c r="J41" s="27"/>
-      <c r="K41" s="27"/>
-      <c r="L41" s="27"/>
-      <c r="M41" s="27"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19"/>
+      <c r="K41" s="19"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="19"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
     </row>
@@ -8880,7 +8880,7 @@
     </row>
     <row r="2" spans="1:15" ht="23" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="22" t="s">
         <v>62</v>
       </c>
       <c r="C2" s="20"/>
@@ -8899,7 +8899,7 @@
     </row>
     <row r="3" spans="1:15" ht="23" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="23" t="s">
         <v>85</v>
       </c>
       <c r="C3" s="20"/>
@@ -8937,21 +8937,21 @@
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="22" t="s">
+      <c r="J5" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
       <c r="O5" s="1"/>
     </row>
     <row r="6" spans="1:15" ht="23" customHeight="1">
@@ -9581,21 +9581,21 @@
     </row>
     <row r="22" spans="1:15" ht="23" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="22"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="21"/>
+      <c r="L22" s="21"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
       <c r="O22" s="1"/>
     </row>
     <row r="23" spans="1:15" ht="23" customHeight="1">
@@ -9608,17 +9608,17 @@
         <v>24</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="23" t="s">
+      <c r="F23" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="23"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
-      <c r="N23" s="23"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="27"/>
+      <c r="M23" s="27"/>
+      <c r="N23" s="27"/>
       <c r="O23" s="1"/>
     </row>
     <row r="24" spans="1:15" ht="23" customHeight="1">
@@ -9631,15 +9631,15 @@
         <v>20</v>
       </c>
       <c r="E24" s="1"/>
-      <c r="F24" s="23"/>
-      <c r="G24" s="23"/>
-      <c r="H24" s="23"/>
-      <c r="I24" s="23"/>
-      <c r="J24" s="23"/>
-      <c r="K24" s="23"/>
-      <c r="L24" s="23"/>
-      <c r="M24" s="23"/>
-      <c r="N24" s="23"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
       <c r="O24" s="1"/>
     </row>
     <row r="25" spans="1:15" ht="23" customHeight="1">
@@ -9705,154 +9705,154 @@
     </row>
     <row r="28" spans="1:15" ht="23" customHeight="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
-      <c r="I28" s="22"/>
-      <c r="J28" s="22"/>
-      <c r="K28" s="22"/>
-      <c r="L28" s="22"/>
-      <c r="M28" s="22"/>
-      <c r="N28" s="22"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="21"/>
+      <c r="K28" s="21"/>
+      <c r="L28" s="21"/>
+      <c r="M28" s="21"/>
+      <c r="N28" s="21"/>
       <c r="O28" s="1"/>
     </row>
     <row r="29" spans="1:15" ht="23" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="24"/>
-      <c r="L29" s="24"/>
-      <c r="M29" s="24"/>
-      <c r="N29" s="24"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="25"/>
+      <c r="K29" s="25"/>
+      <c r="L29" s="25"/>
+      <c r="M29" s="25"/>
+      <c r="N29" s="25"/>
       <c r="O29" s="1"/>
     </row>
     <row r="30" spans="1:15" ht="31" customHeight="1">
       <c r="A30" s="1"/>
-      <c r="B30" s="25" t="s">
+      <c r="B30" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="25"/>
-      <c r="J30" s="25"/>
-      <c r="K30" s="25"/>
-      <c r="L30" s="25"/>
-      <c r="M30" s="25"/>
-      <c r="N30" s="25"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
+      <c r="N30" s="26"/>
       <c r="O30" s="1"/>
     </row>
     <row r="31" spans="1:15" ht="23" customHeight="1">
       <c r="A31" s="1"/>
-      <c r="B31" s="24" t="s">
+      <c r="B31" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="24"/>
-      <c r="H31" s="24"/>
-      <c r="I31" s="24"/>
-      <c r="J31" s="24"/>
-      <c r="K31" s="24"/>
-      <c r="L31" s="24"/>
-      <c r="M31" s="24"/>
-      <c r="N31" s="24"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="25"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="25"/>
+      <c r="M31" s="25"/>
+      <c r="N31" s="25"/>
       <c r="O31" s="1"/>
     </row>
     <row r="32" spans="1:15" ht="23" customHeight="1">
       <c r="A32" s="1"/>
-      <c r="B32" s="24" t="s">
+      <c r="B32" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="24"/>
-      <c r="J32" s="24"/>
-      <c r="K32" s="24"/>
-      <c r="L32" s="24"/>
-      <c r="M32" s="24"/>
-      <c r="N32" s="24"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="25"/>
+      <c r="K32" s="25"/>
+      <c r="L32" s="25"/>
+      <c r="M32" s="25"/>
+      <c r="N32" s="25"/>
       <c r="O32" s="1"/>
     </row>
     <row r="33" spans="1:15" ht="23" customHeight="1">
       <c r="A33" s="1"/>
-      <c r="B33" s="24" t="s">
+      <c r="B33" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="24"/>
-      <c r="J33" s="24"/>
-      <c r="K33" s="24"/>
-      <c r="L33" s="24"/>
-      <c r="M33" s="24"/>
-      <c r="N33" s="24"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="25"/>
+      <c r="K33" s="25"/>
+      <c r="L33" s="25"/>
+      <c r="M33" s="25"/>
+      <c r="N33" s="25"/>
       <c r="O33" s="1"/>
     </row>
     <row r="34" spans="1:15" ht="23" customHeight="1">
       <c r="A34" s="1"/>
-      <c r="B34" s="24" t="s">
+      <c r="B34" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="24"/>
-      <c r="K34" s="24"/>
-      <c r="L34" s="24"/>
-      <c r="M34" s="24"/>
-      <c r="N34" s="24"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="25"/>
+      <c r="K34" s="25"/>
+      <c r="L34" s="25"/>
+      <c r="M34" s="25"/>
+      <c r="N34" s="25"/>
       <c r="O34" s="1"/>
     </row>
     <row r="35" spans="1:15" ht="23" customHeight="1">
       <c r="A35" s="1"/>
-      <c r="B35" s="24" t="s">
+      <c r="B35" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="24"/>
-      <c r="J35" s="24"/>
-      <c r="K35" s="24"/>
-      <c r="L35" s="24"/>
-      <c r="M35" s="24"/>
-      <c r="N35" s="24"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="25"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="25"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="25"/>
+      <c r="K35" s="25"/>
+      <c r="L35" s="25"/>
+      <c r="M35" s="25"/>
+      <c r="N35" s="25"/>
       <c r="O35" s="1"/>
     </row>
     <row r="36" spans="1:15" ht="23" customHeight="1">
@@ -9959,6 +9959,17 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="J5:N5"/>
+    <mergeCell ref="B22:N22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="F23:N24"/>
+    <mergeCell ref="F26:N26"/>
     <mergeCell ref="B33:N33"/>
     <mergeCell ref="B34:N34"/>
     <mergeCell ref="B35:N35"/>
@@ -9967,17 +9978,6 @@
     <mergeCell ref="B30:N30"/>
     <mergeCell ref="B31:N31"/>
     <mergeCell ref="B32:N32"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="F23:N24"/>
-    <mergeCell ref="F26:N26"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="B3:N3"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="J5:N5"/>
-    <mergeCell ref="B22:N22"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11847,47 +11847,47 @@
       </c>
       <c r="F45" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$10:$N$10,1,Q45)+(INDEX(Parameters!$J$10:$N$10,1,Q45+1)-INDEX(Parameters!$J$10:$N$10,1,Q45))*T45,INDEX(Parameters!$D$10:$H$10,1,Q45)+(INDEX(Parameters!$D$10:$H$10,1,Q45+1)-INDEX(Parameters!$D$10:$H$10,1,Q45))*T45)</f>
-        <v>3650</v>
+        <v>4200</v>
       </c>
       <c r="G45" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$11:$N$11,1,R45)+(INDEX(Parameters!$J$11:$N$11,1,R45+1)-INDEX(Parameters!$J$11:$N$11,1,R45))*U45,INDEX(Parameters!$D$11:$H$11,1,Q45)+(INDEX(Parameters!$D$11:$H$11,1,Q45+1)-INDEX(Parameters!$D$11:$H$11,1,Q45))*T45)</f>
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="H45" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$12:$N$12,1,Q45)+(INDEX(Parameters!$J$12:$N$12,1,Q45+1)-INDEX(Parameters!$J$12:$N$12,1,Q45))*T45,INDEX(Parameters!$D$12:$H$12,1,Q45)+(INDEX(Parameters!$D$12:$H$12,1,Q45+1)-INDEX(Parameters!$D$12:$H$12,1,Q45))*T45)</f>
-        <v>0.94</v>
+        <v>0.69</v>
       </c>
       <c r="I45" s="8">
         <f>F45*H45</f>
-        <v>3431</v>
+        <v>2898</v>
       </c>
       <c r="J45" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R45)+(INDEX(Parameters!$J$13:$N$13,1,R45+1)-INDEX(Parameters!$J$13:$N$13,1,R45))*U45,INDEX(Parameters!$D$13:$H$13,1,R45)+(INDEX(Parameters!$D$13:$H$13,1,R45+1)-INDEX(Parameters!$D$13:$H$13,1,R45))*U45)</f>
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="K45" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R45)+(INDEX(Parameters!$D$14:$H$14,1,R45+1)-INDEX(Parameters!$D$14:$H$14,1,R45))*U45)</f>
-        <v>0.34</v>
+        <v>0.6</v>
       </c>
       <c r="L45" s="8">
         <f>I45+J45</f>
-        <v>3681</v>
+        <v>2898</v>
       </c>
       <c r="M45" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S45)+(INDEX(Parameters!$J$17:$N$17,1,S45+1)-INDEX(Parameters!$J$17:$N$17,1,S45))*V45,INDEX(Parameters!$D$17:$H$17,1,S45)+(INDEX(Parameters!$D$17:$H$17,1,S45+1)-INDEX(Parameters!$D$17:$H$17,1,S45))*V45)</f>
-        <v>2100</v>
+        <v>3000</v>
       </c>
       <c r="N45" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$18:$N$18,1,S45)+(INDEX(Parameters!$J$18:$N$18,1,S45+1)-INDEX(Parameters!$J$18:$N$18,1,S45))*V45,INDEX(Parameters!$D$18:$H$18,1,S45)+(INDEX(Parameters!$D$18:$H$18,1,S45+1)-INDEX(Parameters!$D$18:$H$18,1,S45))*V45)</f>
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="O45" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$19:$N$19,1,S45)+(INDEX(Parameters!$J$19:$N$19,1,S45+1)-INDEX(Parameters!$J$19:$N$19,1,S45))*V45,INDEX(Parameters!$D$19:$H$19,1,S45)+(INDEX(Parameters!$D$19:$H$19,1,S45+1)-INDEX(Parameters!$D$19:$H$19,1,S45))*V45)</f>
-        <v>0.92</v>
+        <v>0.68</v>
       </c>
       <c r="P45" s="8">
         <f>M45*O45</f>
-        <v>1932</v>
+        <v>2040.0000000000002</v>
       </c>
       <c r="Q45" s="8">
         <f>MIN(4,MAX(1,INT((1+C45/Parameters!$D$23)*4)+1))</f>
@@ -11933,47 +11933,47 @@
       </c>
       <c r="F46" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$10:$N$10,1,Q46)+(INDEX(Parameters!$J$10:$N$10,1,Q46+1)-INDEX(Parameters!$J$10:$N$10,1,Q46))*T46,INDEX(Parameters!$D$10:$H$10,1,Q46)+(INDEX(Parameters!$D$10:$H$10,1,Q46+1)-INDEX(Parameters!$D$10:$H$10,1,Q46))*T46)</f>
-        <v>3650</v>
+        <v>4200</v>
       </c>
       <c r="G46" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$11:$N$11,1,R46)+(INDEX(Parameters!$J$11:$N$11,1,R46+1)-INDEX(Parameters!$J$11:$N$11,1,R46))*U46,INDEX(Parameters!$D$11:$H$11,1,Q46)+(INDEX(Parameters!$D$11:$H$11,1,Q46+1)-INDEX(Parameters!$D$11:$H$11,1,Q46))*T46)</f>
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="H46" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$12:$N$12,1,Q46)+(INDEX(Parameters!$J$12:$N$12,1,Q46+1)-INDEX(Parameters!$J$12:$N$12,1,Q46))*T46,INDEX(Parameters!$D$12:$H$12,1,Q46)+(INDEX(Parameters!$D$12:$H$12,1,Q46+1)-INDEX(Parameters!$D$12:$H$12,1,Q46))*T46)</f>
-        <v>0.94</v>
+        <v>0.69</v>
       </c>
       <c r="I46" s="8">
         <f>F46*H46</f>
-        <v>3431</v>
+        <v>2898</v>
       </c>
       <c r="J46" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R46)+(INDEX(Parameters!$J$13:$N$13,1,R46+1)-INDEX(Parameters!$J$13:$N$13,1,R46))*U46,INDEX(Parameters!$D$13:$H$13,1,R46)+(INDEX(Parameters!$D$13:$H$13,1,R46+1)-INDEX(Parameters!$D$13:$H$13,1,R46))*U46)</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="K46" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R46)+(INDEX(Parameters!$D$14:$H$14,1,R46+1)-INDEX(Parameters!$D$14:$H$14,1,R46))*U46)</f>
-        <v>0.34499999999999997</v>
+        <v>0.6</v>
       </c>
       <c r="L46" s="8">
         <f>I46+J46</f>
-        <v>4431</v>
+        <v>2898</v>
       </c>
       <c r="M46" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S46)+(INDEX(Parameters!$J$17:$N$17,1,S46+1)-INDEX(Parameters!$J$17:$N$17,1,S46))*V46,INDEX(Parameters!$D$17:$H$17,1,S46)+(INDEX(Parameters!$D$17:$H$17,1,S46+1)-INDEX(Parameters!$D$17:$H$17,1,S46))*V46)</f>
-        <v>2850</v>
+        <v>3750</v>
       </c>
       <c r="N46" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$18:$N$18,1,S46)+(INDEX(Parameters!$J$18:$N$18,1,S46+1)-INDEX(Parameters!$J$18:$N$18,1,S46))*V46,INDEX(Parameters!$D$18:$H$18,1,S46)+(INDEX(Parameters!$D$18:$H$18,1,S46+1)-INDEX(Parameters!$D$18:$H$18,1,S46))*V46)</f>
-        <v>0.24</v>
+        <v>0.215</v>
       </c>
       <c r="O46" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$19:$N$19,1,S46)+(INDEX(Parameters!$J$19:$N$19,1,S46+1)-INDEX(Parameters!$J$19:$N$19,1,S46))*V46,INDEX(Parameters!$D$19:$H$19,1,S46)+(INDEX(Parameters!$D$19:$H$19,1,S46+1)-INDEX(Parameters!$D$19:$H$19,1,S46))*V46)</f>
-        <v>0.89</v>
+        <v>0.65</v>
       </c>
       <c r="P46" s="8">
         <f>M46*O46</f>
-        <v>2536.5</v>
+        <v>2437.5</v>
       </c>
       <c r="Q46" s="8">
         <f>MIN(4,MAX(1,INT((1+C46/Parameters!$D$23)*4)+1))</f>
@@ -12019,47 +12019,47 @@
       </c>
       <c r="F47" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$10:$N$10,1,Q47)+(INDEX(Parameters!$J$10:$N$10,1,Q47+1)-INDEX(Parameters!$J$10:$N$10,1,Q47))*T47,INDEX(Parameters!$D$10:$H$10,1,Q47)+(INDEX(Parameters!$D$10:$H$10,1,Q47+1)-INDEX(Parameters!$D$10:$H$10,1,Q47))*T47)</f>
-        <v>3650</v>
+        <v>4200</v>
       </c>
       <c r="G47" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$11:$N$11,1,R47)+(INDEX(Parameters!$J$11:$N$11,1,R47+1)-INDEX(Parameters!$J$11:$N$11,1,R47))*U47,INDEX(Parameters!$D$11:$H$11,1,Q47)+(INDEX(Parameters!$D$11:$H$11,1,Q47+1)-INDEX(Parameters!$D$11:$H$11,1,Q47))*T47)</f>
-        <v>0.08</v>
+        <v>0.3</v>
       </c>
       <c r="H47" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$12:$N$12,1,Q47)+(INDEX(Parameters!$J$12:$N$12,1,Q47+1)-INDEX(Parameters!$J$12:$N$12,1,Q47))*T47,INDEX(Parameters!$D$12:$H$12,1,Q47)+(INDEX(Parameters!$D$12:$H$12,1,Q47+1)-INDEX(Parameters!$D$12:$H$12,1,Q47))*T47)</f>
-        <v>0.94</v>
+        <v>0.69</v>
       </c>
       <c r="I47" s="8">
         <f>F47*H47</f>
-        <v>3431</v>
+        <v>2898</v>
       </c>
       <c r="J47" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R47)+(INDEX(Parameters!$J$13:$N$13,1,R47+1)-INDEX(Parameters!$J$13:$N$13,1,R47))*U47,INDEX(Parameters!$D$13:$H$13,1,R47)+(INDEX(Parameters!$D$13:$H$13,1,R47+1)-INDEX(Parameters!$D$13:$H$13,1,R47))*U47)</f>
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="K47" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R47)+(INDEX(Parameters!$D$14:$H$14,1,R47+1)-INDEX(Parameters!$D$14:$H$14,1,R47))*U47)</f>
-        <v>0.35</v>
+        <v>0.6</v>
       </c>
       <c r="L47" s="8">
         <f>I47+J47</f>
-        <v>5181</v>
+        <v>2898</v>
       </c>
       <c r="M47" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S47)+(INDEX(Parameters!$J$17:$N$17,1,S47+1)-INDEX(Parameters!$J$17:$N$17,1,S47))*V47,INDEX(Parameters!$D$17:$H$17,1,S47)+(INDEX(Parameters!$D$17:$H$17,1,S47+1)-INDEX(Parameters!$D$17:$H$17,1,S47))*V47)</f>
-        <v>3600</v>
+        <v>4500</v>
       </c>
       <c r="N47" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$18:$N$18,1,S47)+(INDEX(Parameters!$J$18:$N$18,1,S47+1)-INDEX(Parameters!$J$18:$N$18,1,S47))*V47,INDEX(Parameters!$D$18:$H$18,1,S47)+(INDEX(Parameters!$D$18:$H$18,1,S47+1)-INDEX(Parameters!$D$18:$H$18,1,S47))*V47)</f>
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="O47" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$19:$N$19,1,S47)+(INDEX(Parameters!$J$19:$N$19,1,S47+1)-INDEX(Parameters!$J$19:$N$19,1,S47))*V47,INDEX(Parameters!$D$19:$H$19,1,S47)+(INDEX(Parameters!$D$19:$H$19,1,S47+1)-INDEX(Parameters!$D$19:$H$19,1,S47))*V47)</f>
-        <v>0.86</v>
+        <v>0.62</v>
       </c>
       <c r="P47" s="8">
         <f>M47*O47</f>
-        <v>3096</v>
+        <v>2790</v>
       </c>
       <c r="Q47" s="8">
         <f>MIN(4,MAX(1,INT((1+C47/Parameters!$D$23)*4)+1))</f>
@@ -12105,47 +12105,47 @@
       </c>
       <c r="F48" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$10:$N$10,1,Q48)+(INDEX(Parameters!$J$10:$N$10,1,Q48+1)-INDEX(Parameters!$J$10:$N$10,1,Q48))*T48,INDEX(Parameters!$D$10:$H$10,1,Q48)+(INDEX(Parameters!$D$10:$H$10,1,Q48+1)-INDEX(Parameters!$D$10:$H$10,1,Q48))*T48)</f>
-        <v>3650</v>
+        <v>4200</v>
       </c>
       <c r="G48" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$11:$N$11,1,R48)+(INDEX(Parameters!$J$11:$N$11,1,R48+1)-INDEX(Parameters!$J$11:$N$11,1,R48))*U48,INDEX(Parameters!$D$11:$H$11,1,Q48)+(INDEX(Parameters!$D$11:$H$11,1,Q48+1)-INDEX(Parameters!$D$11:$H$11,1,Q48))*T48)</f>
-        <v>0.08</v>
+        <v>0.35</v>
       </c>
       <c r="H48" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$12:$N$12,1,Q48)+(INDEX(Parameters!$J$12:$N$12,1,Q48+1)-INDEX(Parameters!$J$12:$N$12,1,Q48))*T48,INDEX(Parameters!$D$12:$H$12,1,Q48)+(INDEX(Parameters!$D$12:$H$12,1,Q48+1)-INDEX(Parameters!$D$12:$H$12,1,Q48))*T48)</f>
-        <v>0.94</v>
+        <v>0.69</v>
       </c>
       <c r="I48" s="8">
         <f>F48*H48</f>
-        <v>3431</v>
+        <v>2898</v>
       </c>
       <c r="J48" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R48)+(INDEX(Parameters!$J$13:$N$13,1,R48+1)-INDEX(Parameters!$J$13:$N$13,1,R48))*U48,INDEX(Parameters!$D$13:$H$13,1,R48)+(INDEX(Parameters!$D$13:$H$13,1,R48+1)-INDEX(Parameters!$D$13:$H$13,1,R48))*U48)</f>
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="K48" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R48)+(INDEX(Parameters!$D$14:$H$14,1,R48+1)-INDEX(Parameters!$D$14:$H$14,1,R48))*U48)</f>
-        <v>0.35499999999999998</v>
+        <v>0.6</v>
       </c>
       <c r="L48" s="8">
         <f>I48+J48</f>
-        <v>5931</v>
+        <v>2898</v>
       </c>
       <c r="M48" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S48)+(INDEX(Parameters!$J$17:$N$17,1,S48+1)-INDEX(Parameters!$J$17:$N$17,1,S48))*V48,INDEX(Parameters!$D$17:$H$17,1,S48)+(INDEX(Parameters!$D$17:$H$17,1,S48+1)-INDEX(Parameters!$D$17:$H$17,1,S48))*V48)</f>
-        <v>4350</v>
+        <v>5250</v>
       </c>
       <c r="N48" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$18:$N$18,1,S48)+(INDEX(Parameters!$J$18:$N$18,1,S48+1)-INDEX(Parameters!$J$18:$N$18,1,S48))*V48,INDEX(Parameters!$D$18:$H$18,1,S48)+(INDEX(Parameters!$D$18:$H$18,1,S48+1)-INDEX(Parameters!$D$18:$H$18,1,S48))*V48)</f>
-        <v>0.26</v>
+        <v>0.22500000000000001</v>
       </c>
       <c r="O48" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$19:$N$19,1,S48)+(INDEX(Parameters!$J$19:$N$19,1,S48+1)-INDEX(Parameters!$J$19:$N$19,1,S48))*V48,INDEX(Parameters!$D$19:$H$19,1,S48)+(INDEX(Parameters!$D$19:$H$19,1,S48+1)-INDEX(Parameters!$D$19:$H$19,1,S48))*V48)</f>
-        <v>0.83000000000000007</v>
+        <v>0.59000000000000008</v>
       </c>
       <c r="P48" s="8">
         <f>M48*O48</f>
-        <v>3610.5000000000005</v>
+        <v>3097.5000000000005</v>
       </c>
       <c r="Q48" s="8">
         <f>MIN(4,MAX(1,INT((1+C48/Parameters!$D$23)*4)+1))</f>
@@ -12191,47 +12191,47 @@
       </c>
       <c r="F49" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$10:$N$10,1,Q49)+(INDEX(Parameters!$J$10:$N$10,1,Q49+1)-INDEX(Parameters!$J$10:$N$10,1,Q49))*T49,INDEX(Parameters!$D$10:$H$10,1,Q49)+(INDEX(Parameters!$D$10:$H$10,1,Q49+1)-INDEX(Parameters!$D$10:$H$10,1,Q49))*T49)</f>
-        <v>3650</v>
+        <v>4200</v>
       </c>
       <c r="G49" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$11:$N$11,1,R49)+(INDEX(Parameters!$J$11:$N$11,1,R49+1)-INDEX(Parameters!$J$11:$N$11,1,R49))*U49,INDEX(Parameters!$D$11:$H$11,1,Q49)+(INDEX(Parameters!$D$11:$H$11,1,Q49+1)-INDEX(Parameters!$D$11:$H$11,1,Q49))*T49)</f>
-        <v>0.08</v>
+        <v>0.4</v>
       </c>
       <c r="H49" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$12:$N$12,1,Q49)+(INDEX(Parameters!$J$12:$N$12,1,Q49+1)-INDEX(Parameters!$J$12:$N$12,1,Q49))*T49,INDEX(Parameters!$D$12:$H$12,1,Q49)+(INDEX(Parameters!$D$12:$H$12,1,Q49+1)-INDEX(Parameters!$D$12:$H$12,1,Q49))*T49)</f>
-        <v>0.94</v>
+        <v>0.69</v>
       </c>
       <c r="I49" s="8">
         <f>F49*H49</f>
-        <v>3431</v>
+        <v>2898</v>
       </c>
       <c r="J49" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$13:$N$13,1,R49)+(INDEX(Parameters!$J$13:$N$13,1,R49+1)-INDEX(Parameters!$J$13:$N$13,1,R49))*U49,INDEX(Parameters!$D$13:$H$13,1,R49)+(INDEX(Parameters!$D$13:$H$13,1,R49+1)-INDEX(Parameters!$D$13:$H$13,1,R49))*U49)</f>
-        <v>3250</v>
+        <v>0</v>
       </c>
       <c r="K49" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",Parameters!$L$14,INDEX(Parameters!$D$14:$H$14,1,R49)+(INDEX(Parameters!$D$14:$H$14,1,R49+1)-INDEX(Parameters!$D$14:$H$14,1,R49))*U49)</f>
-        <v>0.36</v>
+        <v>0.6</v>
       </c>
       <c r="L49" s="8">
         <f>I49+J49</f>
-        <v>6681</v>
+        <v>2898</v>
       </c>
       <c r="M49" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$17:$N$17,1,S49)+(INDEX(Parameters!$J$17:$N$17,1,S49+1)-INDEX(Parameters!$J$17:$N$17,1,S49))*V49,INDEX(Parameters!$D$17:$H$17,1,S49)+(INDEX(Parameters!$D$17:$H$17,1,S49+1)-INDEX(Parameters!$D$17:$H$17,1,S49))*V49)</f>
-        <v>5100</v>
+        <v>6000</v>
       </c>
       <c r="N49" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$18:$N$18,1,S49)+(INDEX(Parameters!$J$18:$N$18,1,S49+1)-INDEX(Parameters!$J$18:$N$18,1,S49))*V49,INDEX(Parameters!$D$18:$H$18,1,S49)+(INDEX(Parameters!$D$18:$H$18,1,S49+1)-INDEX(Parameters!$D$18:$H$18,1,S49))*V49)</f>
-        <v>0.27</v>
+        <v>0.23</v>
       </c>
       <c r="O49" s="8">
         <f>IF('HSC Sweep'!$C$4="Type-B",INDEX(Parameters!$J$19:$N$19,1,S49)+(INDEX(Parameters!$J$19:$N$19,1,S49+1)-INDEX(Parameters!$J$19:$N$19,1,S49))*V49,INDEX(Parameters!$D$19:$H$19,1,S49)+(INDEX(Parameters!$D$19:$H$19,1,S49+1)-INDEX(Parameters!$D$19:$H$19,1,S49))*V49)</f>
-        <v>0.8</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="P49" s="8">
         <f>M49*O49</f>
-        <v>4080</v>
+        <v>3360.0000000000005</v>
       </c>
       <c r="Q49" s="8">
         <f>MIN(4,MAX(1,INT((1+C49/Parameters!$D$23)*4)+1))</f>
@@ -12413,23 +12413,23 @@
       </c>
       <c r="C55" s="15">
         <f t="shared" si="5"/>
-        <v>182.5</v>
+        <v>210</v>
       </c>
       <c r="D55" s="15">
         <f t="shared" si="6"/>
-        <v>182.5</v>
+        <v>210</v>
       </c>
       <c r="E55" s="15">
         <f t="shared" si="7"/>
-        <v>182.5</v>
+        <v>210</v>
       </c>
       <c r="F55" s="15">
         <f t="shared" si="8"/>
-        <v>182.5</v>
+        <v>210</v>
       </c>
       <c r="G55" s="15">
         <f t="shared" si="9"/>
-        <v>182.5</v>
+        <v>210</v>
       </c>
       <c r="H55" s="8"/>
       <c r="I55" s="8"/>
@@ -12453,23 +12453,23 @@
       </c>
       <c r="C56" s="15">
         <f t="shared" si="5"/>
-        <v>360.62</v>
+        <v>420</v>
       </c>
       <c r="D56" s="15">
         <f t="shared" si="6"/>
-        <v>360.62</v>
+        <v>420</v>
       </c>
       <c r="E56" s="15">
         <f t="shared" si="7"/>
-        <v>360.62</v>
+        <v>420</v>
       </c>
       <c r="F56" s="15">
         <f t="shared" si="8"/>
-        <v>360.62</v>
+        <v>420</v>
       </c>
       <c r="G56" s="15">
         <f t="shared" si="9"/>
-        <v>360.62</v>
+        <v>420</v>
       </c>
       <c r="H56" s="8"/>
       <c r="I56" s="8"/>
@@ -12493,23 +12493,23 @@
       </c>
       <c r="C57" s="15">
         <f t="shared" si="5"/>
-        <v>532.16999999999996</v>
+        <v>630</v>
       </c>
       <c r="D57" s="15">
         <f t="shared" si="6"/>
-        <v>532.16999999999996</v>
+        <v>630</v>
       </c>
       <c r="E57" s="15">
         <f t="shared" si="7"/>
-        <v>532.16999999999996</v>
+        <v>630</v>
       </c>
       <c r="F57" s="15">
         <f t="shared" si="8"/>
-        <v>532.16999999999996</v>
+        <v>630</v>
       </c>
       <c r="G57" s="15">
         <f t="shared" si="9"/>
-        <v>532.16999999999996</v>
+        <v>630</v>
       </c>
       <c r="H57" s="8"/>
       <c r="I57" s="8"/>
@@ -12533,23 +12533,23 @@
       </c>
       <c r="C58" s="15">
         <f t="shared" si="5"/>
-        <v>703.72</v>
+        <v>840</v>
       </c>
       <c r="D58" s="15">
         <f t="shared" si="6"/>
-        <v>703.72</v>
+        <v>840</v>
       </c>
       <c r="E58" s="15">
         <f t="shared" si="7"/>
-        <v>703.72</v>
+        <v>840</v>
       </c>
       <c r="F58" s="15">
         <f t="shared" si="8"/>
-        <v>703.72</v>
+        <v>840</v>
       </c>
       <c r="G58" s="15">
         <f t="shared" si="9"/>
-        <v>703.72</v>
+        <v>840</v>
       </c>
       <c r="H58" s="8"/>
       <c r="I58" s="8"/>
@@ -12573,23 +12573,23 @@
       </c>
       <c r="C59" s="15">
         <f t="shared" si="5"/>
-        <v>875.27</v>
+        <v>984.9</v>
       </c>
       <c r="D59" s="15">
         <f t="shared" si="6"/>
-        <v>875.27</v>
+        <v>1050</v>
       </c>
       <c r="E59" s="15">
         <f t="shared" si="7"/>
-        <v>875.27</v>
+        <v>1050</v>
       </c>
       <c r="F59" s="15">
         <f t="shared" si="8"/>
-        <v>875.27</v>
+        <v>1050</v>
       </c>
       <c r="G59" s="15">
         <f t="shared" si="9"/>
-        <v>875.27</v>
+        <v>1050</v>
       </c>
       <c r="H59" s="8"/>
       <c r="I59" s="8"/>
@@ -12613,23 +12613,23 @@
       </c>
       <c r="C60" s="15">
         <f t="shared" si="5"/>
-        <v>1046.82</v>
+        <v>1129.8</v>
       </c>
       <c r="D60" s="15">
         <f t="shared" si="6"/>
-        <v>1046.82</v>
+        <v>1194.9000000000001</v>
       </c>
       <c r="E60" s="15">
         <f t="shared" si="7"/>
-        <v>1046.82</v>
+        <v>1260</v>
       </c>
       <c r="F60" s="15">
         <f t="shared" si="8"/>
-        <v>1046.82</v>
+        <v>1260</v>
       </c>
       <c r="G60" s="15">
         <f t="shared" si="9"/>
-        <v>1046.82</v>
+        <v>1260</v>
       </c>
       <c r="H60" s="8"/>
       <c r="I60" s="8"/>
@@ -12653,23 +12653,23 @@
       </c>
       <c r="C61" s="15">
         <f t="shared" si="5"/>
-        <v>1220.8699999999999</v>
+        <v>1274.6999999999998</v>
       </c>
       <c r="D61" s="15">
         <f t="shared" si="6"/>
-        <v>1223.3699999999999</v>
+        <v>1339.8</v>
       </c>
       <c r="E61" s="15">
         <f t="shared" si="7"/>
-        <v>1218.3699999999999</v>
+        <v>1404.9</v>
       </c>
       <c r="F61" s="15">
         <f t="shared" si="8"/>
-        <v>1218.3699999999999</v>
+        <v>1470</v>
       </c>
       <c r="G61" s="15">
         <f t="shared" si="9"/>
-        <v>1218.3699999999999</v>
+        <v>1470</v>
       </c>
       <c r="H61" s="8"/>
       <c r="I61" s="8"/>
@@ -12693,23 +12693,23 @@
       </c>
       <c r="C62" s="15">
         <f t="shared" si="5"/>
-        <v>1404.92</v>
+        <v>1419.6</v>
       </c>
       <c r="D62" s="15">
         <f t="shared" si="6"/>
-        <v>1444.92</v>
+        <v>1484.7</v>
       </c>
       <c r="E62" s="15">
         <f t="shared" si="7"/>
-        <v>1477.42</v>
+        <v>1549.8000000000002</v>
       </c>
       <c r="F62" s="15">
         <f t="shared" si="8"/>
-        <v>1502.42</v>
+        <v>1614.9</v>
       </c>
       <c r="G62" s="15">
         <f t="shared" si="9"/>
-        <v>1519.92</v>
+        <v>1680</v>
       </c>
       <c r="H62" s="8"/>
       <c r="I62" s="8"/>
@@ -12733,23 +12733,23 @@
       </c>
       <c r="C63" s="15">
         <f t="shared" si="5"/>
-        <v>1588.97</v>
+        <v>1564.5</v>
       </c>
       <c r="D63" s="15">
         <f t="shared" si="6"/>
-        <v>1666.47</v>
+        <v>1629.6</v>
       </c>
       <c r="E63" s="15">
         <f t="shared" si="7"/>
-        <v>1736.47</v>
+        <v>1694.7</v>
       </c>
       <c r="F63" s="15">
         <f t="shared" si="8"/>
-        <v>1798.97</v>
+        <v>1759.8000000000002</v>
       </c>
       <c r="G63" s="15">
         <f t="shared" si="9"/>
-        <v>1853.97</v>
+        <v>1824.9</v>
       </c>
       <c r="H63" s="8"/>
       <c r="I63" s="8"/>
@@ -12773,23 +12773,23 @@
       </c>
       <c r="C64" s="15">
         <f t="shared" si="5"/>
-        <v>1773.02</v>
+        <v>1709.4</v>
       </c>
       <c r="D64" s="15">
         <f t="shared" si="6"/>
-        <v>1888.02</v>
+        <v>1774.5</v>
       </c>
       <c r="E64" s="15">
         <f t="shared" si="7"/>
-        <v>1995.52</v>
+        <v>1839.6</v>
       </c>
       <c r="F64" s="15">
         <f t="shared" si="8"/>
-        <v>2095.52</v>
+        <v>1904.7</v>
       </c>
       <c r="G64" s="15">
         <f t="shared" si="9"/>
-        <v>2188.02</v>
+        <v>1969.8</v>
       </c>
       <c r="H64" s="8"/>
       <c r="I64" s="8"/>
@@ -12813,23 +12813,23 @@
       </c>
       <c r="C65" s="15">
         <f t="shared" si="5"/>
-        <v>1957.0700000000002</v>
+        <v>1854.3000000000002</v>
       </c>
       <c r="D65" s="15">
         <f t="shared" si="6"/>
-        <v>2109.5700000000002</v>
+        <v>1919.4</v>
       </c>
       <c r="E65" s="15">
         <f t="shared" si="7"/>
-        <v>2254.5700000000002</v>
+        <v>1984.5</v>
       </c>
       <c r="F65" s="15">
         <f t="shared" si="8"/>
-        <v>2392.0700000000002</v>
+        <v>2049.6000000000004</v>
       </c>
       <c r="G65" s="15">
         <f t="shared" si="9"/>
-        <v>2522.0700000000006</v>
+        <v>2114.6999999999998</v>
       </c>
       <c r="H65" s="8"/>
       <c r="I65" s="8"/>
@@ -12853,23 +12853,23 @@
       </c>
       <c r="C66" s="15">
         <f t="shared" si="5"/>
-        <v>2141.12</v>
+        <v>1999.1999999999998</v>
       </c>
       <c r="D66" s="15">
         <f t="shared" si="6"/>
-        <v>2331.12</v>
+        <v>2064.3000000000002</v>
       </c>
       <c r="E66" s="15">
         <f t="shared" si="7"/>
-        <v>2513.62</v>
+        <v>2129.4</v>
       </c>
       <c r="F66" s="15">
         <f t="shared" si="8"/>
-        <v>2688.62</v>
+        <v>2194.5</v>
       </c>
       <c r="G66" s="15">
         <f t="shared" si="9"/>
-        <v>2856.12</v>
+        <v>2259.6</v>
       </c>
       <c r="H66" s="8"/>
       <c r="I66" s="8"/>
@@ -12893,23 +12893,23 @@
       </c>
       <c r="C67" s="15">
         <f t="shared" si="5"/>
-        <v>2325.17</v>
+        <v>2144.1000000000004</v>
       </c>
       <c r="D67" s="15">
         <f t="shared" si="6"/>
-        <v>2552.67</v>
+        <v>2209.1999999999998</v>
       </c>
       <c r="E67" s="15">
         <f t="shared" si="7"/>
-        <v>2772.67</v>
+        <v>2274.3000000000002</v>
       </c>
       <c r="F67" s="15">
         <f t="shared" si="8"/>
-        <v>2985.17</v>
+        <v>2339.4</v>
       </c>
       <c r="G67" s="15">
         <f t="shared" si="9"/>
-        <v>3190.17</v>
+        <v>2404.5</v>
       </c>
       <c r="H67" s="8"/>
       <c r="I67" s="8"/>
@@ -12933,23 +12933,23 @@
       </c>
       <c r="C68" s="15">
         <f t="shared" si="5"/>
-        <v>2509.2199999999998</v>
+        <v>2289</v>
       </c>
       <c r="D68" s="15">
         <f t="shared" si="6"/>
-        <v>2774.22</v>
+        <v>2354.1</v>
       </c>
       <c r="E68" s="15">
         <f t="shared" si="7"/>
-        <v>3031.72</v>
+        <v>2419.1999999999998</v>
       </c>
       <c r="F68" s="15">
         <f t="shared" si="8"/>
-        <v>3281.72</v>
+        <v>2484.3000000000002</v>
       </c>
       <c r="G68" s="15">
         <f t="shared" si="9"/>
-        <v>3524.22</v>
+        <v>2549.3999999999996</v>
       </c>
       <c r="H68" s="8"/>
       <c r="I68" s="8"/>
@@ -12973,23 +12973,23 @@
       </c>
       <c r="C69" s="15">
         <f t="shared" si="5"/>
-        <v>2693.27</v>
+        <v>2433.9</v>
       </c>
       <c r="D69" s="15">
         <f t="shared" si="6"/>
-        <v>2995.77</v>
+        <v>2499</v>
       </c>
       <c r="E69" s="15">
         <f t="shared" si="7"/>
-        <v>3290.77</v>
+        <v>2564.1000000000004</v>
       </c>
       <c r="F69" s="15">
         <f t="shared" si="8"/>
-        <v>3578.27</v>
+        <v>2629.2</v>
       </c>
       <c r="G69" s="15">
         <f t="shared" si="9"/>
-        <v>3858.27</v>
+        <v>2694.3</v>
       </c>
       <c r="H69" s="8"/>
       <c r="I69" s="8"/>
@@ -13013,23 +13013,23 @@
       </c>
       <c r="C70" s="15">
         <f t="shared" si="5"/>
-        <v>2877.32</v>
+        <v>2578.8000000000002</v>
       </c>
       <c r="D70" s="15">
         <f t="shared" si="6"/>
-        <v>3217.32</v>
+        <v>2643.9</v>
       </c>
       <c r="E70" s="15">
         <f t="shared" si="7"/>
-        <v>3549.82</v>
+        <v>2709</v>
       </c>
       <c r="F70" s="15">
         <f t="shared" si="8"/>
-        <v>3874.8200000000006</v>
+        <v>2774.1000000000004</v>
       </c>
       <c r="G70" s="15">
         <f t="shared" si="9"/>
-        <v>4192.3200000000006</v>
+        <v>2839.2</v>
       </c>
       <c r="H70" s="8"/>
       <c r="I70" s="8"/>
@@ -13053,23 +13053,23 @@
       </c>
       <c r="C71" s="15">
         <f t="shared" si="5"/>
-        <v>3061.37</v>
+        <v>2723.7</v>
       </c>
       <c r="D71" s="15">
         <f t="shared" si="6"/>
-        <v>3438.87</v>
+        <v>2788.8</v>
       </c>
       <c r="E71" s="15">
         <f t="shared" si="7"/>
-        <v>3808.87</v>
+        <v>2853.9</v>
       </c>
       <c r="F71" s="15">
         <f t="shared" si="8"/>
-        <v>4171.37</v>
+        <v>2919</v>
       </c>
       <c r="G71" s="15">
         <f t="shared" si="9"/>
-        <v>4526.37</v>
+        <v>2984.1</v>
       </c>
       <c r="H71" s="8"/>
       <c r="I71" s="8"/>
@@ -13093,23 +13093,23 @@
       </c>
       <c r="C72" s="15">
         <f t="shared" si="5"/>
-        <v>3245.42</v>
+        <v>2868.6</v>
       </c>
       <c r="D72" s="15">
         <f t="shared" si="6"/>
-        <v>3660.42</v>
+        <v>2933.7</v>
       </c>
       <c r="E72" s="15">
         <f t="shared" si="7"/>
-        <v>4067.92</v>
+        <v>2998.8</v>
       </c>
       <c r="F72" s="15">
         <f t="shared" si="8"/>
-        <v>4467.92</v>
+        <v>3063.9</v>
       </c>
       <c r="G72" s="15">
         <f t="shared" si="9"/>
-        <v>4860.42</v>
+        <v>3129</v>
       </c>
       <c r="H72" s="8"/>
       <c r="I72" s="8"/>
@@ -13133,23 +13133,23 @@
       </c>
       <c r="C73" s="15">
         <f t="shared" si="5"/>
-        <v>3429.47</v>
+        <v>3013.5</v>
       </c>
       <c r="D73" s="15">
         <f t="shared" si="6"/>
-        <v>3881.97</v>
+        <v>3078.6</v>
       </c>
       <c r="E73" s="15">
         <f t="shared" si="7"/>
-        <v>4326.9699999999993</v>
+        <v>3143.7</v>
       </c>
       <c r="F73" s="15">
         <f t="shared" si="8"/>
-        <v>4764.4699999999993</v>
+        <v>3208.8</v>
       </c>
       <c r="G73" s="15">
         <f t="shared" si="9"/>
-        <v>5194.4699999999993</v>
+        <v>3273.8999999999996</v>
       </c>
       <c r="H73" s="8"/>
       <c r="I73" s="8"/>
@@ -13173,23 +13173,23 @@
       </c>
       <c r="C74" s="15">
         <f t="shared" si="5"/>
-        <v>3613.52</v>
+        <v>3158.4</v>
       </c>
       <c r="D74" s="15">
         <f t="shared" si="6"/>
-        <v>4103.5200000000004</v>
+        <v>3223.5</v>
       </c>
       <c r="E74" s="15">
         <f t="shared" si="7"/>
-        <v>4586.0200000000004</v>
+        <v>3288.6</v>
       </c>
       <c r="F74" s="15">
         <f t="shared" si="8"/>
-        <v>5061.0200000000004</v>
+        <v>3353.7</v>
       </c>
       <c r="G74" s="15">
         <f t="shared" si="9"/>
-        <v>5528.52</v>
+        <v>3418.8</v>
       </c>
       <c r="H74" s="8"/>
       <c r="I74" s="8"/>

</xml_diff>